<commit_message>
exp: finish the edu+1 computation
</commit_message>
<xml_diff>
--- a/MLD01e_Results/SummaryTable_ModelPerformance.xlsx
+++ b/MLD01e_Results/SummaryTable_ModelPerformance.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10824"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ccceaaab575c7926/MLD01_Article/MLD01e_Results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="57" documentId="8_{DA289BF3-DC6D-474B-8054-3BCD6735358D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6858C826-B600-0640-8A2E-41608DBC833A}"/>
+  <xr:revisionPtr revIDLastSave="166" documentId="8_{DA289BF3-DC6D-474B-8054-3BCD6735358D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9051CEFB-F40C-495D-93BC-02184FAAA663}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="34560" windowHeight="21600" xr2:uid="{16EB2B38-9B61-B846-8886-60DE5182E9FB}"/>
+    <workbookView xWindow="33780" yWindow="255" windowWidth="14325" windowHeight="14730" xr2:uid="{16EB2B38-9B61-B846-8886-60DE5182E9FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -171,7 +171,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -179,13 +179,14 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="10" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -525,14 +526,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C4C94BE-B4AA-A947-925C-1C2708BC0BA7}">
   <dimension ref="A1:M18"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15.9" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="21.5" style="1" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="10.83203125" style="1"/>
+    <col min="2" max="2" width="10.85546875" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="10.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A1" s="5" t="s">
         <v>28</v>
       </c>
@@ -549,7 +550,7 @@
       <c r="L1" s="5"/>
       <c r="M1" s="5"/>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.45">
       <c r="B2" s="5" t="s">
         <v>16</v>
       </c>
@@ -569,7 +570,7 @@
       <c r="L2" s="5"/>
       <c r="M2" s="5"/>
     </row>
-    <row r="3" spans="1:13" ht="49" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:13" ht="49" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>20</v>
       </c>
@@ -598,7 +599,7 @@
       </c>
       <c r="M3" s="5"/>
     </row>
-    <row r="4" spans="1:13" ht="17" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>19</v>
       </c>
@@ -639,578 +640,578 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="17" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:13" ht="16.75" x14ac:dyDescent="0.45">
       <c r="A5" s="2" t="s">
         <v>2</v>
       </c>
       <c r="B5" s="1">
         <v>500</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D5" s="1">
         <v>1000</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="3" t="s">
         <v>22</v>
       </c>
       <c r="F5" s="1">
-        <v>1000</v>
-      </c>
-      <c r="G5" s="4" t="s">
+        <v>500</v>
+      </c>
+      <c r="G5" s="3" t="s">
         <v>22</v>
       </c>
       <c r="H5" s="1">
         <v>1000</v>
       </c>
-      <c r="I5" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="J5" s="1">
+      <c r="I5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="J5" s="4">
+        <v>2000</v>
+      </c>
+      <c r="K5" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="L5" s="4">
         <v>1000</v>
       </c>
-      <c r="K5" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="L5" s="1">
-        <v>1000</v>
-      </c>
       <c r="M5" s="4" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="17" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:13" ht="16.75" x14ac:dyDescent="0.45">
       <c r="A6" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="1">
         <v>0.01</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D6" s="1">
         <v>0.05</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="3" t="s">
         <v>22</v>
       </c>
       <c r="F6" s="1">
         <v>0.01</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="G6" s="3" t="s">
         <v>22</v>
       </c>
       <c r="H6" s="1">
         <v>0.01</v>
       </c>
-      <c r="I6" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="J6" s="1">
+      <c r="I6" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="J6" s="4">
         <v>0.01</v>
       </c>
       <c r="K6" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="L6" s="1">
-        <v>0.01</v>
+      <c r="L6" s="4">
+        <v>0.05</v>
       </c>
       <c r="M6" s="4" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="17" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:13" ht="16.75" x14ac:dyDescent="0.45">
       <c r="A7" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B7" s="1">
         <v>8</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D7" s="1">
         <v>16</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="3" t="s">
         <v>22</v>
       </c>
       <c r="F7" s="1">
         <v>16</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="G7" s="3" t="s">
         <v>22</v>
       </c>
       <c r="H7" s="1">
         <v>16</v>
       </c>
-      <c r="I7" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="J7" s="1">
+      <c r="I7" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="J7" s="4">
         <v>16</v>
       </c>
       <c r="K7" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="L7" s="1">
+      <c r="L7" s="4">
         <v>16</v>
       </c>
       <c r="M7" s="4" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="17" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:13" ht="16.75" x14ac:dyDescent="0.45">
       <c r="A8" s="2" t="s">
         <v>5</v>
       </c>
       <c r="B8" s="1">
         <v>0.7</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D8" s="1">
         <v>0.9</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="3" t="s">
         <v>22</v>
       </c>
       <c r="F8" s="1">
         <v>0.9</v>
       </c>
-      <c r="G8" s="4" t="s">
+      <c r="G8" s="3" t="s">
         <v>22</v>
       </c>
       <c r="H8" s="1">
-        <v>0.7</v>
-      </c>
-      <c r="I8" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="J8" s="1">
-        <v>0.7</v>
+        <v>0.9</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="J8" s="4">
+        <v>0.8</v>
       </c>
       <c r="K8" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="L8" s="1">
-        <v>0.7</v>
+      <c r="L8" s="4">
+        <v>1</v>
       </c>
       <c r="M8" s="4" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:13" ht="17" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:13" ht="15.9" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="2" t="s">
         <v>6</v>
       </c>
       <c r="B9" s="1">
         <v>0.7</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D9" s="1">
         <v>1</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E9" s="3" t="s">
         <v>22</v>
       </c>
       <c r="F9" s="1">
-        <v>0.9</v>
-      </c>
-      <c r="G9" s="4" t="s">
+        <v>0.7</v>
+      </c>
+      <c r="G9" s="3" t="s">
         <v>22</v>
       </c>
       <c r="H9" s="1">
         <v>0.9</v>
       </c>
-      <c r="I9" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="J9" s="1">
+      <c r="I9" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="J9" s="4">
+        <v>0.7</v>
+      </c>
+      <c r="K9" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="L9" s="4">
         <v>0.9</v>
       </c>
-      <c r="K9" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="L9" s="1">
-        <v>0.9</v>
-      </c>
       <c r="M9" s="4" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:13" ht="17" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:13" ht="16.75" x14ac:dyDescent="0.45">
       <c r="A10" s="2" t="s">
         <v>7</v>
       </c>
       <c r="B10" s="1">
         <v>5</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D10" s="1">
         <v>1</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="E10" s="3" t="s">
         <v>22</v>
       </c>
       <c r="F10" s="1">
         <v>1</v>
       </c>
-      <c r="G10" s="4" t="s">
+      <c r="G10" s="3" t="s">
         <v>22</v>
       </c>
       <c r="H10" s="1">
         <v>1</v>
       </c>
-      <c r="I10" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="J10" s="1">
-        <v>1</v>
+      <c r="I10" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="J10" s="4">
+        <v>2</v>
       </c>
       <c r="K10" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="L10" s="1">
-        <v>1</v>
+      <c r="L10" s="4">
+        <v>2</v>
       </c>
       <c r="M10" s="4" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="18" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" ht="16.75" x14ac:dyDescent="0.45">
       <c r="A11" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="3">
+      <c r="B11" s="6">
         <v>0.76002599999999998</v>
       </c>
-      <c r="C11" s="3">
+      <c r="C11" s="6">
         <v>0.62966900000000003</v>
       </c>
-      <c r="D11" s="3">
-        <v>0.89626600000000001</v>
-      </c>
-      <c r="E11" s="3">
-        <v>0.42306300000000002</v>
-      </c>
-      <c r="F11" s="3">
-        <v>0.86185999999999996</v>
-      </c>
-      <c r="G11" s="3">
-        <v>0.57391000000000003</v>
-      </c>
-      <c r="H11" s="3">
-        <v>0.84586899999999998</v>
-      </c>
-      <c r="I11" s="3">
-        <v>0.63233399999999995</v>
-      </c>
-      <c r="J11" s="3">
-        <v>0.83333299999999999</v>
-      </c>
-      <c r="K11" s="3">
-        <v>0.66493800000000003</v>
-      </c>
-      <c r="L11" s="3">
-        <v>0.86220600000000003</v>
-      </c>
-      <c r="M11" s="3">
-        <v>0.69943100000000002</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" ht="18" x14ac:dyDescent="0.25">
+      <c r="D11" s="6">
+        <v>0.89635200000000004</v>
+      </c>
+      <c r="E11" s="6">
+        <v>0.423842</v>
+      </c>
+      <c r="F11" s="6">
+        <v>0.86410699999999996</v>
+      </c>
+      <c r="G11" s="6">
+        <v>0.56145500000000004</v>
+      </c>
+      <c r="H11" s="6">
+        <v>0.84828899999999996</v>
+      </c>
+      <c r="I11" s="6">
+        <v>0.63268199999999997</v>
+      </c>
+      <c r="J11" s="6">
+        <v>0.835063</v>
+      </c>
+      <c r="K11" s="6">
+        <v>0.66026499999999999</v>
+      </c>
+      <c r="L11" s="6">
+        <v>0.86497299999999999</v>
+      </c>
+      <c r="M11" s="6">
+        <v>0.69519699999999995</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" ht="16.75" x14ac:dyDescent="0.45">
       <c r="A12" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="3">
+      <c r="B12" s="6">
         <v>0.71449099999999999</v>
       </c>
-      <c r="C12" s="3">
+      <c r="C12" s="6">
         <v>0.57620800000000005</v>
       </c>
-      <c r="D12" s="3">
-        <v>0.92546700000000004</v>
-      </c>
-      <c r="E12" s="3">
-        <v>0.94779199999999997</v>
-      </c>
-      <c r="F12" s="3">
-        <v>0.69155199999999994</v>
-      </c>
-      <c r="G12" s="3">
-        <v>0.29641099999999998</v>
-      </c>
-      <c r="H12" s="3">
-        <v>0.70396199999999998</v>
-      </c>
-      <c r="I12" s="3">
-        <v>0.36678899999999998</v>
-      </c>
-      <c r="J12" s="3">
-        <v>0.74268400000000001</v>
-      </c>
-      <c r="K12" s="3">
-        <v>0.47590300000000002</v>
-      </c>
-      <c r="L12" s="3">
-        <v>0.79163399999999995</v>
-      </c>
-      <c r="M12" s="3">
-        <v>0.557508</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" ht="18" x14ac:dyDescent="0.25">
+      <c r="D12" s="6">
+        <v>0.92563700000000004</v>
+      </c>
+      <c r="E12" s="6">
+        <v>0.94847700000000001</v>
+      </c>
+      <c r="F12" s="6">
+        <v>0.68916599999999995</v>
+      </c>
+      <c r="G12" s="6">
+        <v>0.29296699999999998</v>
+      </c>
+      <c r="H12" s="6">
+        <v>0.70903499999999997</v>
+      </c>
+      <c r="I12" s="6">
+        <v>0.36417699999999997</v>
+      </c>
+      <c r="J12" s="6">
+        <v>0.74754799999999999</v>
+      </c>
+      <c r="K12" s="6">
+        <v>0.469252</v>
+      </c>
+      <c r="L12" s="6">
+        <v>0.80035400000000001</v>
+      </c>
+      <c r="M12" s="6">
+        <v>0.54492300000000005</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" ht="16.75" x14ac:dyDescent="0.45">
       <c r="A13" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="3">
+      <c r="B13" s="6">
         <v>0.71821400000000002</v>
       </c>
-      <c r="C13" s="3">
+      <c r="C13" s="6">
         <v>0.47065000000000001</v>
       </c>
-      <c r="D13" s="3">
-        <v>0.962391</v>
-      </c>
-      <c r="E13" s="3">
-        <v>0.38088100000000003</v>
-      </c>
-      <c r="F13" s="3">
-        <v>0.62136199999999997</v>
-      </c>
-      <c r="G13" s="3">
-        <v>0.71819599999999995</v>
-      </c>
-      <c r="H13" s="3">
-        <v>0.62450300000000003</v>
-      </c>
-      <c r="I13" s="3">
-        <v>0.64387700000000003</v>
-      </c>
-      <c r="J13" s="3">
-        <v>0.71496499999999996</v>
-      </c>
-      <c r="K13" s="3">
-        <v>0.55164100000000005</v>
-      </c>
-      <c r="L13" s="3">
-        <v>0.78162299999999996</v>
-      </c>
-      <c r="M13" s="3">
-        <v>0.45404</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" ht="18" x14ac:dyDescent="0.25">
+      <c r="D13" s="6">
+        <v>0.96229399999999998</v>
+      </c>
+      <c r="E13" s="6">
+        <v>0.38164999999999999</v>
+      </c>
+      <c r="F13" s="6">
+        <v>0.64641300000000002</v>
+      </c>
+      <c r="G13" s="6">
+        <v>0.75720500000000002</v>
+      </c>
+      <c r="H13" s="6">
+        <v>0.63131499999999996</v>
+      </c>
+      <c r="I13" s="6">
+        <v>0.66428100000000001</v>
+      </c>
+      <c r="J13" s="6">
+        <v>0.71413499999999996</v>
+      </c>
+      <c r="K13" s="6">
+        <v>0.56568700000000005</v>
+      </c>
+      <c r="L13" s="6">
+        <v>0.77869699999999997</v>
+      </c>
+      <c r="M13" s="6">
+        <v>0.47428300000000001</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" ht="16.75" x14ac:dyDescent="0.45">
       <c r="A14" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="3">
+      <c r="B14" s="6">
         <v>0.71619699999999997</v>
       </c>
-      <c r="C14" s="3">
+      <c r="C14" s="6">
         <v>0.51598200000000005</v>
       </c>
-      <c r="D14" s="3">
-        <v>0.94355599999999995</v>
-      </c>
-      <c r="E14" s="3">
-        <v>0.54174900000000004</v>
-      </c>
-      <c r="F14" s="3">
-        <v>0.65421300000000004</v>
-      </c>
-      <c r="G14" s="3">
-        <v>0.41479100000000002</v>
-      </c>
-      <c r="H14" s="3">
-        <v>0.66140399999999999</v>
-      </c>
-      <c r="I14" s="3">
-        <v>0.45915</v>
-      </c>
-      <c r="J14" s="3">
-        <v>0.72825399999999996</v>
-      </c>
-      <c r="K14" s="3">
-        <v>0.50529800000000002</v>
-      </c>
-      <c r="L14" s="3">
-        <v>0.78648600000000002</v>
-      </c>
-      <c r="M14" s="3">
-        <v>0.49341699999999999</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" ht="18" x14ac:dyDescent="0.25">
+      <c r="D14" s="6">
+        <v>0.94359800000000005</v>
+      </c>
+      <c r="E14" s="6">
+        <v>0.54248200000000002</v>
+      </c>
+      <c r="F14" s="6">
+        <v>0.66688400000000003</v>
+      </c>
+      <c r="G14" s="6">
+        <v>0.42094399999999998</v>
+      </c>
+      <c r="H14" s="6">
+        <v>0.66742000000000001</v>
+      </c>
+      <c r="I14" s="6">
+        <v>0.46670499999999998</v>
+      </c>
+      <c r="J14" s="6">
+        <v>0.73017299999999996</v>
+      </c>
+      <c r="K14" s="6">
+        <v>0.50859799999999999</v>
+      </c>
+      <c r="L14" s="6">
+        <v>0.78921300000000005</v>
+      </c>
+      <c r="M14" s="6">
+        <v>0.50065499999999996</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" ht="16.75" x14ac:dyDescent="0.45">
       <c r="A15" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B15" s="3">
+      <c r="B15" s="6">
         <v>1.0266000000000001E-2</v>
       </c>
-      <c r="C15" s="3">
+      <c r="C15" s="6">
         <v>1.5776999999999999E-2</v>
       </c>
-      <c r="D15" s="3">
-        <v>7.6099999999999996E-3</v>
-      </c>
-      <c r="E15" s="3">
-        <v>3.9328000000000002E-2</v>
-      </c>
-      <c r="F15" s="3">
-        <v>6.2820000000000003E-3</v>
-      </c>
-      <c r="G15" s="3">
-        <v>7.2137999999999994E-2</v>
-      </c>
-      <c r="H15" s="3">
-        <v>7.1729999999999997E-3</v>
-      </c>
-      <c r="I15" s="3">
-        <v>7.1178000000000005E-2</v>
-      </c>
-      <c r="J15" s="3">
-        <v>6.9150000000000001E-3</v>
-      </c>
-      <c r="K15" s="3">
-        <v>3.7347999999999999E-2</v>
-      </c>
-      <c r="L15" s="3">
-        <v>1.0933E-2</v>
-      </c>
-      <c r="M15" s="3">
-        <v>3.6602000000000003E-2</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13" ht="18" x14ac:dyDescent="0.25">
+      <c r="D15" s="6">
+        <v>8.0400000000000003E-3</v>
+      </c>
+      <c r="E15" s="6">
+        <v>3.9461000000000003E-2</v>
+      </c>
+      <c r="F15" s="6">
+        <v>6.4019999999999997E-3</v>
+      </c>
+      <c r="G15" s="6">
+        <v>4.7718000000000003E-2</v>
+      </c>
+      <c r="H15" s="6">
+        <v>7.6049999999999998E-3</v>
+      </c>
+      <c r="I15" s="6">
+        <v>5.3837000000000003E-2</v>
+      </c>
+      <c r="J15" s="6">
+        <v>6.548E-3</v>
+      </c>
+      <c r="K15" s="6">
+        <v>2.9704999999999999E-2</v>
+      </c>
+      <c r="L15" s="6">
+        <v>8.3560000000000006E-3</v>
+      </c>
+      <c r="M15" s="6">
+        <v>3.2621999999999998E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" ht="16.75" x14ac:dyDescent="0.45">
       <c r="A16" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B16" s="3">
+      <c r="B16" s="6">
         <v>1.6917999999999999E-2</v>
       </c>
-      <c r="C16" s="3">
+      <c r="C16" s="6">
         <v>2.8830000000000001E-2</v>
       </c>
-      <c r="D16" s="3">
-        <v>4.3270000000000001E-3</v>
-      </c>
-      <c r="E16" s="3">
-        <v>1.3358E-2</v>
-      </c>
-      <c r="F16" s="3">
-        <v>1.8539E-2</v>
-      </c>
-      <c r="G16" s="3">
-        <v>2.4115000000000001E-2</v>
-      </c>
-      <c r="H16" s="3">
-        <v>2.0240999999999999E-2</v>
-      </c>
-      <c r="I16" s="3">
-        <v>4.8566999999999999E-2</v>
-      </c>
-      <c r="J16" s="3">
-        <v>1.1842999999999999E-2</v>
-      </c>
-      <c r="K16" s="3">
-        <v>3.1109999999999999E-2</v>
-      </c>
-      <c r="L16" s="3">
-        <v>2.0822E-2</v>
-      </c>
-      <c r="M16" s="3">
-        <v>4.9169999999999998E-2</v>
-      </c>
-    </row>
-    <row r="17" spans="1:13" ht="18" x14ac:dyDescent="0.25">
+      <c r="D16" s="6">
+        <v>5.0850000000000001E-3</v>
+      </c>
+      <c r="E16" s="6">
+        <v>1.4747E-2</v>
+      </c>
+      <c r="F16" s="6">
+        <v>1.8688E-2</v>
+      </c>
+      <c r="G16" s="6">
+        <v>1.5261E-2</v>
+      </c>
+      <c r="H16" s="6">
+        <v>2.3411999999999999E-2</v>
+      </c>
+      <c r="I16" s="6">
+        <v>3.2506E-2</v>
+      </c>
+      <c r="J16" s="6">
+        <v>1.5003000000000001E-2</v>
+      </c>
+      <c r="K16" s="6">
+        <v>2.8726999999999999E-2</v>
+      </c>
+      <c r="L16" s="6">
+        <v>1.7815999999999999E-2</v>
+      </c>
+      <c r="M16" s="6">
+        <v>5.1640999999999999E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" ht="16.75" x14ac:dyDescent="0.45">
       <c r="A17" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B17" s="3">
+      <c r="B17" s="6">
         <v>1.2329E-2</v>
       </c>
-      <c r="C17" s="3">
+      <c r="C17" s="6">
         <v>5.4297999999999999E-2</v>
       </c>
-      <c r="D17" s="3">
-        <v>6.5040000000000002E-3</v>
-      </c>
-      <c r="E17" s="3">
-        <v>4.7653000000000001E-2</v>
-      </c>
-      <c r="F17" s="3">
-        <v>2.8147999999999999E-2</v>
-      </c>
-      <c r="G17" s="3">
-        <v>0.12717700000000001</v>
-      </c>
-      <c r="H17" s="3">
-        <v>2.8417999999999999E-2</v>
-      </c>
-      <c r="I17" s="3">
-        <v>0.10756599999999999</v>
-      </c>
-      <c r="J17" s="3">
-        <v>2.7146E-2</v>
-      </c>
-      <c r="K17" s="3">
-        <v>9.9138000000000004E-2</v>
-      </c>
-      <c r="L17" s="3">
-        <v>1.6389000000000001E-2</v>
-      </c>
-      <c r="M17" s="3">
-        <v>8.3462999999999996E-2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13" ht="18" x14ac:dyDescent="0.25">
+      <c r="D17" s="6">
+        <v>6.241E-3</v>
+      </c>
+      <c r="E17" s="6">
+        <v>4.9021000000000002E-2</v>
+      </c>
+      <c r="F17" s="6">
+        <v>2.1739999999999999E-2</v>
+      </c>
+      <c r="G17" s="6">
+        <v>8.1100000000000005E-2</v>
+      </c>
+      <c r="H17" s="6">
+        <v>2.7217000000000002E-2</v>
+      </c>
+      <c r="I17" s="6">
+        <v>8.0347000000000002E-2</v>
+      </c>
+      <c r="J17" s="6">
+        <v>2.2818000000000001E-2</v>
+      </c>
+      <c r="K17" s="6">
+        <v>8.4609000000000004E-2</v>
+      </c>
+      <c r="L17" s="6">
+        <v>1.6601000000000001E-2</v>
+      </c>
+      <c r="M17" s="6">
+        <v>8.0381999999999995E-2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" ht="16.75" x14ac:dyDescent="0.45">
       <c r="A18" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B18" s="3">
+      <c r="B18" s="6">
         <v>1.0099E-2</v>
       </c>
-      <c r="C18" s="3">
+      <c r="C18" s="6">
         <v>2.9172E-2</v>
       </c>
-      <c r="D18" s="3">
-        <v>4.2110000000000003E-3</v>
-      </c>
-      <c r="E18" s="3">
-        <v>4.7143999999999998E-2</v>
-      </c>
-      <c r="F18" s="3">
-        <v>1.8253999999999999E-2</v>
-      </c>
-      <c r="G18" s="3">
-        <v>1.5864E-2</v>
-      </c>
-      <c r="H18" s="3">
-        <v>1.8079999999999999E-2</v>
-      </c>
-      <c r="I18" s="3">
-        <v>1.9837E-2</v>
-      </c>
-      <c r="J18" s="3">
-        <v>1.4638999999999999E-2</v>
-      </c>
-      <c r="K18" s="3">
-        <v>2.5270000000000001E-2</v>
-      </c>
-      <c r="L18" s="3">
-        <v>1.5994000000000001E-2</v>
-      </c>
-      <c r="M18" s="3">
-        <v>2.5426000000000001E-2</v>
+      <c r="D18" s="6">
+        <v>4.4149999999999997E-3</v>
+      </c>
+      <c r="E18" s="6">
+        <v>4.7839E-2</v>
+      </c>
+      <c r="F18" s="6">
+        <v>1.6098999999999999E-2</v>
+      </c>
+      <c r="G18" s="6">
+        <v>1.5748999999999999E-2</v>
+      </c>
+      <c r="H18" s="6">
+        <v>1.7024000000000001E-2</v>
+      </c>
+      <c r="I18" s="6">
+        <v>1.839E-2</v>
+      </c>
+      <c r="J18" s="6">
+        <v>1.2259000000000001E-2</v>
+      </c>
+      <c r="K18" s="6">
+        <v>2.0145E-2</v>
+      </c>
+      <c r="L18" s="6">
+        <v>1.2403000000000001E-2</v>
+      </c>
+      <c r="M18" s="6">
+        <v>3.3647000000000003E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>